<commit_message>
vers 6.10 aggiornamento dati Lord Rayleigh
</commit_message>
<xml_diff>
--- a/Dati/L'azoto di Lord Rayleigh.xlsx
+++ b/Dati/L'azoto di Lord Rayleigh.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MODUNIVAR\Shiny\Dati\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\RSTUDIOAPPLICATIVI\Modunivar\Dati\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97003465-B4BB-462D-9E60-1C30EF7B6FE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E2DDED1-AE5A-4145-85CA-F77660D23311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
+    <sheet name="Dataset" sheetId="1" r:id="rId1"/>
+    <sheet name="Presentazione dell'esperimento" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="125725"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="6">
   <si>
     <t>Origine</t>
   </si>
@@ -38,11 +39,20 @@
   <si>
     <t>Azoto</t>
   </si>
+  <si>
+    <t>Origine del gas</t>
+  </si>
+  <si>
+    <t>massa di N2 (g)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.00000"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -79,12 +89,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normale" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -97,6 +114,262 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>161924</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>542924</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4BAAB584-4FD4-7012-8F61-D8042D167CE7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2200275" y="161924"/>
+          <a:ext cx="13925549" cy="2152651"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100"/>
+            <a:t>L'esperimento condotto da Lord Rayleigh (John William Strutt) alla fine del 1800 gli valse </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>il Premio Nobel per la Fisica nel 1904. </a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Le prove di Rayleigh erano in origine</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100"/>
+            <a:t>mirate </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>alla determinazione della quantità di azoto nell'aria, ma </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100"/>
+            <a:t>portarono</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100" baseline="0"/>
+            <a:t> a</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100"/>
+            <a:t>lla scoperta dell'Argon.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100"/>
+            <a:t>L'esperimento di Rayleigh consisteva</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100" baseline="0"/>
+            <a:t> nel</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100"/>
+            <a:t> confronto di due metodi diversi per ottenere azoto:</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100"/>
+            <a:t>Metodo 1: isolamento dell'azoto dall'aria: R. fece passare aria in un tubo di rame rovente per rimuovere l'ossigeno (che forma ossido di rame,</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100" baseline="0"/>
+            <a:t> CuO e CO2</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100"/>
+            <a:t>), e poi attraverso una soluzione alcalina per rimuovere l'anidride carbonica.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100"/>
+            <a:t>Il gas residuo è azoto puro proveniente al</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100" baseline="0"/>
+            <a:t> 100%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100"/>
+            <a:t> dall'aria.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100"/>
+            <a:t>Metodo 2: ottenimento</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100" baseline="0"/>
+            <a:t> dell'a</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100"/>
+            <a:t>zoto dal suo ossido N2O: con lo stesso processo di riscaldamento e gorgogliamento in soluzione alcalina, a partire dal protossido di azoto, si ottiene una miscela di gas costituita da azoto e ossigeno in rapporto</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100" baseline="0"/>
+            <a:t> 2 a 1, e si ricava così uno "standard" di azoto </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100"/>
+            <a:t>puro.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100"/>
+            <a:t>Rayleigh osservò con</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100" baseline="0"/>
+            <a:t> queste e altre prove (condotte con diversi altri composti azotati) </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100"/>
+            <a:t>che l'azoto atmosferico (Metodo 1) ha una densità (massa per unità di volume) maggiore rispetto all'azoto standard</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100" baseline="0"/>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100"/>
+            <a:t>"chimico" (Metodo 2).</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100"/>
+            <a:t>La piccola differenza di massa nei due gas fu interpretata ammettendo che l'azoto atmosferico non fosse puro, ma che contenesse un gas sconosciuto più pesante che non veniva eliminato nel processo di preparazione allestito per</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100" baseline="0"/>
+            <a:t> l'azoto</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100"/>
+            <a:t>.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100"/>
+            <a:t>In collaborazione con William Ramsay, Rayleigh  quindi isolò questo gas sconosciuto, che si rivelò essere un elemento nuovo, chimicamente inerte, che chiamarono Argon (dal greco argos, "inattivo").</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100"/>
+            <a:t>Questo esperimento è celebre perché dimostrò che misurazioni di alta precisione e la capacità di mettere in evidenza piccole differenze di massa potevano portare a scoperte scientifiche fondamentali, e .</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="it-IT" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -363,9 +636,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -373,83 +646,83 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="4">
         <v>2.3100999999999998</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="4">
         <v>2.3100100000000001</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="4">
         <v>2.3102399999999998</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="4">
         <v>2.3100999999999998</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="4">
         <v>2.3102800000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="4">
         <v>2.2989000000000002</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="4">
         <v>2.2981600000000002</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="4">
         <v>2.3018200000000002</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="4">
         <v>2.2986900000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="4">
         <v>2.2993999999999999</v>
       </c>
     </row>
@@ -457,4 +730,107 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CAC6630-E56A-43C3-95A0-AD7E59C90887}">
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.140625" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" style="2" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3">
+        <v>2.3100999999999998</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3">
+        <v>2.3100100000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3">
+        <v>2.3102399999999998</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="3">
+        <v>2.3100999999999998</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="3">
+        <v>2.3102800000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" s="3">
+        <v>2.2989000000000002</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" s="3">
+        <v>2.2981600000000002</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" s="3">
+        <v>2.3018200000000002</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" s="3">
+        <v>2.2986900000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" s="3">
+        <v>2.2993999999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>